<commit_message>
Build Business Tangent deck as PPTX and PDF from the model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MCV8azwG9F4KBgd2vtZi4v
</commit_message>
<xml_diff>
--- a/business-tangent-fpo/model/KAP_FPO_Model.xlsx
+++ b/business-tangent-fpo/model/KAP_FPO_Model.xlsx
@@ -13,13 +13,14 @@
     <sheet sheetId="7" name="Budget" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Targets" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="Checks" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Sensitivity" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="331">
   <si>
     <t>Case data (as given in the case)</t>
   </si>
@@ -969,7 +970,49 @@
     <t>Fund capital covers what is lent out (0 if yes)</t>
   </si>
   <si>
+    <t>Sensitivity base equals Unit_Econ cover</t>
+  </si>
+  <si>
     <t>Federation covers its running cost (0 if yes)</t>
+  </si>
+  <si>
+    <t>Year 5 cost cover under stress (produce-linked income scales with the driver)</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>What changes</t>
+  </si>
+  <si>
+    <t>Base case</t>
+  </si>
+  <si>
+    <t>Model as built</t>
+  </si>
+  <si>
+    <t>Only 39% of members sell (SRIJAN level)</t>
+  </si>
+  <si>
+    <t>[S9]</t>
+  </si>
+  <si>
+    <t>Prices 10% lower</t>
+  </si>
+  <si>
+    <t>Produce margins fall in proportion</t>
+  </si>
+  <si>
+    <t>Maize yield 4.0 t/ha</t>
+  </si>
+  <si>
+    <t>[S11] state average</t>
+  </si>
+  <si>
+    <t>Flood year: vegetables lose 1 of 1.5 seasons</t>
+  </si>
+  <si>
+    <t>Kharif vegetable season lost</t>
   </si>
 </sst>
 </file>
@@ -1694,6 +1737,121 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="52" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C3" s="20">
+        <f>((Unit_Econ!$D$12+Unit_Econ!$D$13+Unit_Econ!$D$16)*1+Unit_Econ!$D$14)/Unit_Econ!$D$25</f>
+        <v>0.97517660156</v>
+      </c>
+      <c r="D3" s="20">
+        <f>(Unit_Econ!$F$12*1+(Unit_Econ!$F$14+Unit_Econ!$F$15+Unit_Econ!$F$16))/Unit_Econ!$F$25</f>
+        <v>0.92406454272</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="C4" s="20">
+        <f>((Unit_Econ!$D$12+Unit_Econ!$D$13+Unit_Econ!$D$16)*0.39/Assumptions!$C$8+Unit_Econ!$D$14)/Unit_Econ!$D$25</f>
+        <v>0.82086786123</v>
+      </c>
+      <c r="D4" s="20">
+        <f>(Unit_Econ!$F$12*0.39/Assumptions!$D$8+(Unit_Econ!$F$14+Unit_Econ!$F$15+Unit_Econ!$F$16))/Unit_Econ!$F$25</f>
+        <v>0.85222462706</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C5" s="20">
+        <f>((Unit_Econ!$D$12+Unit_Econ!$D$13+Unit_Econ!$D$16)*0.9+Unit_Econ!$D$14)/Unit_Econ!$D$25</f>
+        <v>0.90503626505</v>
+      </c>
+      <c r="D5" s="20">
+        <f>(Unit_Econ!$F$12*0.9+(Unit_Econ!$F$14+Unit_Econ!$F$15+Unit_Econ!$F$16))/Unit_Econ!$F$25</f>
+        <v>0.87018460597</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C6" s="20">
+        <f>((Unit_Econ!$D$12+Unit_Econ!$D$13+Unit_Econ!$D$16)*4/Assumptions!$C$10+Unit_Econ!$D$14)/Unit_Econ!$D$25</f>
+        <v>0.89724289432</v>
+      </c>
+      <c r="D6" s="20">
+        <f>(Unit_Econ!$F$12*1+(Unit_Econ!$F$14+Unit_Econ!$F$15+Unit_Econ!$F$16))/Unit_Econ!$F$25</f>
+        <v>0.92406454272</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C7" s="20">
+        <f>((Unit_Econ!$D$12+Unit_Econ!$D$13+Unit_Econ!$D$16)*1+Unit_Econ!$D$14)/Unit_Econ!$D$25</f>
+        <v>0.97517660156</v>
+      </c>
+      <c r="D7" s="20">
+        <f>(Unit_Econ!$F$12*1/1.5+(Unit_Econ!$F$14+Unit_Econ!$F$15+Unit_Econ!$F$16))/Unit_Econ!$F$25</f>
+        <v>0.74446475358</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>330</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E46"/>
@@ -4447,7 +4605,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
@@ -4556,11 +4714,24 @@
         <v>316</v>
       </c>
       <c r="C9" s="27">
-        <f>MAX(0,1-Federation!$C$24)</f>
+        <f>ABS(Sensitivity!$C$3-Unit_Econ!$D$26)+ABS(Sensitivity!$D$3-Unit_Econ!$F$26)</f>
         <v>0</v>
       </c>
       <c r="D9" s="28" t="str">
         <f>IF(ABS(C9)&lt;0.001,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="C10" s="27">
+        <f>MAX(0,1-Federation!$C$24)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="28" t="str">
+        <f>IF(ABS(C10)&lt;0.001,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>

</xml_diff>